<commit_message>
Größeres Dialogfenster (+nur noch eins)
</commit_message>
<xml_diff>
--- a/Länder-Fakten.xlsx
+++ b/Länder-Fakten.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\LasseDorn\Repos\Quiz-World\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC87A8E1-06F3-4209-8210-E617C0A0A9EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2CC03EF-B3F1-4650-980B-BA36726EF2DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20715" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4257,9 +4257,6 @@
     <t>Chile</t>
   </si>
   <si>
-    <t>Volksrepublik China</t>
-  </si>
-  <si>
     <t>Costa Rica</t>
   </si>
   <si>
@@ -4479,9 +4476,6 @@
     <t>Mexiko</t>
   </si>
   <si>
-    <t>Republik Moldau</t>
-  </si>
-  <si>
     <t>Mongolei</t>
   </si>
   <si>
@@ -4539,9 +4533,6 @@
     <t>Pakistan</t>
   </si>
   <si>
-    <t>Palästinensische Autonomiebehörde</t>
-  </si>
-  <si>
     <t>Palau</t>
   </si>
   <si>
@@ -4731,10 +4722,19 @@
     <t>Zentralafrikanische Republik</t>
   </si>
   <si>
-    <t>Republik Zypern</t>
-  </si>
-  <si>
     <t>Land A-Z</t>
+  </si>
+  <si>
+    <t>Zypern</t>
+  </si>
+  <si>
+    <t>China</t>
+  </si>
+  <si>
+    <t>Moldawien</t>
+  </si>
+  <si>
+    <t>Palästina</t>
   </si>
 </sst>
 </file>
@@ -5276,24 +5276,24 @@
   <dimension ref="A1:M203"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.06640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="30.86328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.9296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.73046875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.86328125" customWidth="1"/>
-    <col min="7" max="7" width="23.73046875" customWidth="1"/>
-    <col min="8" max="8" width="13.73046875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15.9296875" customWidth="1"/>
-    <col min="10" max="10" width="16.9296875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.19921875" style="7" customWidth="1"/>
-    <col min="12" max="12" width="76.1328125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.53125" style="11" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.3984375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.86328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.73046875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.73046875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.46484375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15.53125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13" style="7" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="77.265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.796875" style="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
-        <v>1553</v>
+        <v>1549</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -6547,7 +6547,7 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A33" s="16" t="s">
-        <v>1394</v>
+        <v>1551</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>164</v>
@@ -6586,7 +6586,7 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A34" s="16" t="s">
-        <v>1395</v>
+        <v>1394</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>56</v>
@@ -6625,7 +6625,7 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A35" s="16" t="s">
-        <v>1396</v>
+        <v>1395</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>179</v>
@@ -6666,7 +6666,7 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A36" s="16" t="s">
-        <v>1397</v>
+        <v>1396</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>189</v>
@@ -6705,7 +6705,7 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A37" s="16" t="s">
-        <v>1398</v>
+        <v>1397</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>194</v>
@@ -6744,7 +6744,7 @@
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A38" s="16" t="s">
-        <v>1399</v>
+        <v>1398</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>46</v>
@@ -6783,7 +6783,7 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A39" s="16" t="s">
-        <v>1400</v>
+        <v>1399</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>56</v>
@@ -6861,7 +6861,7 @@
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A41" s="16" t="s">
-        <v>1401</v>
+        <v>1400</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>212</v>
@@ -6900,7 +6900,7 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A42" s="16" t="s">
-        <v>1402</v>
+        <v>1401</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>56</v>
@@ -6939,7 +6939,7 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A43" s="16" t="s">
-        <v>1403</v>
+        <v>1402</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>113</v>
@@ -6978,7 +6978,7 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A44" s="16" t="s">
-        <v>1404</v>
+        <v>1403</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>226</v>
@@ -7017,7 +7017,7 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A45" s="16" t="s">
-        <v>1405</v>
+        <v>1404</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>230</v>
@@ -7056,7 +7056,7 @@
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A46" s="16" t="s">
-        <v>1406</v>
+        <v>1405</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>235</v>
@@ -7095,7 +7095,7 @@
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A47" s="16" t="s">
-        <v>1407</v>
+        <v>1406</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>297</v>
@@ -7134,7 +7134,7 @@
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A48" s="16" t="s">
-        <v>1408</v>
+        <v>1407</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>304</v>
@@ -7173,7 +7173,7 @@
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A49" s="16" t="s">
-        <v>1409</v>
+        <v>1408</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>113</v>
@@ -7212,7 +7212,7 @@
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A50" s="16" t="s">
-        <v>1410</v>
+        <v>1409</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>113</v>
@@ -7251,7 +7251,7 @@
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A51" s="16" t="s">
-        <v>1411</v>
+        <v>1410</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>46</v>
@@ -7290,7 +7290,7 @@
     </row>
     <row r="52" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A52" s="16" t="s">
-        <v>1412</v>
+        <v>1411</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>323</v>
@@ -7329,7 +7329,7 @@
     </row>
     <row r="53" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A53" s="16" t="s">
-        <v>1413</v>
+        <v>1412</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>46</v>
@@ -7368,7 +7368,7 @@
     </row>
     <row r="54" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A54" s="16" t="s">
-        <v>1414</v>
+        <v>1413</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>46</v>
@@ -7407,7 +7407,7 @@
     </row>
     <row r="55" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A55" s="16" t="s">
-        <v>1415</v>
+        <v>1414</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>340</v>
@@ -7446,7 +7446,7 @@
     </row>
     <row r="56" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A56" s="16" t="s">
-        <v>1416</v>
+        <v>1415</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>184</v>
@@ -7487,7 +7487,7 @@
     </row>
     <row r="57" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A57" s="16" t="s">
-        <v>1417</v>
+        <v>1416</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>56</v>
@@ -7526,7 +7526,7 @@
     </row>
     <row r="58" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A58" s="16" t="s">
-        <v>1418</v>
+        <v>1417</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>113</v>
@@ -7565,7 +7565,7 @@
     </row>
     <row r="59" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A59" s="16" t="s">
-        <v>1419</v>
+        <v>1418</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>41</v>
@@ -7604,7 +7604,7 @@
     </row>
     <row r="60" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A60" s="16" t="s">
-        <v>1420</v>
+        <v>1419</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>46</v>
@@ -7643,7 +7643,7 @@
     </row>
     <row r="61" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A61" s="16" t="s">
-        <v>1421</v>
+        <v>1420</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>364</v>
@@ -7682,7 +7682,7 @@
     </row>
     <row r="62" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A62" s="16" t="s">
-        <v>1422</v>
+        <v>1421</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>56</v>
@@ -7721,7 +7721,7 @@
     </row>
     <row r="63" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A63" s="16" t="s">
-        <v>1423</v>
+        <v>1422</v>
       </c>
       <c r="B63" s="3" t="s">
         <v>375</v>
@@ -7760,7 +7760,7 @@
     </row>
     <row r="64" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A64" s="16" t="s">
-        <v>1424</v>
+        <v>1423</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>381</v>
@@ -7799,7 +7799,7 @@
     </row>
     <row r="65" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A65" s="16" t="s">
-        <v>1425</v>
+        <v>1424</v>
       </c>
       <c r="B65" s="3" t="s">
         <v>387</v>
@@ -7838,7 +7838,7 @@
     </row>
     <row r="66" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A66" s="16" t="s">
-        <v>1426</v>
+        <v>1425</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>393</v>
@@ -7877,7 +7877,7 @@
     </row>
     <row r="67" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A67" s="16" t="s">
-        <v>1427</v>
+        <v>1426</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>399</v>
@@ -7916,7 +7916,7 @@
     </row>
     <row r="68" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A68" s="16" t="s">
-        <v>1428</v>
+        <v>1427</v>
       </c>
       <c r="B68" s="3" t="s">
         <v>403</v>
@@ -7955,7 +7955,7 @@
     </row>
     <row r="69" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A69" s="16" t="s">
-        <v>1429</v>
+        <v>1428</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>410</v>
@@ -7994,7 +7994,7 @@
     </row>
     <row r="70" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A70" s="16" t="s">
-        <v>1430</v>
+        <v>1429</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>416</v>
@@ -8033,7 +8033,7 @@
     </row>
     <row r="71" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A71" s="16" t="s">
-        <v>1431</v>
+        <v>1430</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>46</v>
@@ -8072,7 +8072,7 @@
     </row>
     <row r="72" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A72" s="16" t="s">
-        <v>1432</v>
+        <v>1431</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>426</v>
@@ -8111,7 +8111,7 @@
     </row>
     <row r="73" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A73" s="16" t="s">
-        <v>1433</v>
+        <v>1432</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>14</v>
@@ -8150,7 +8150,7 @@
     </row>
     <row r="74" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A74" s="16" t="s">
-        <v>1434</v>
+        <v>1433</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>14</v>
@@ -8189,7 +8189,7 @@
     </row>
     <row r="75" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A75" s="16" t="s">
-        <v>1435</v>
+        <v>1434</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>440</v>
@@ -8228,7 +8228,7 @@
     </row>
     <row r="76" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A76" s="16" t="s">
-        <v>1436</v>
+        <v>1435</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>446</v>
@@ -8267,7 +8267,7 @@
     </row>
     <row r="77" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A77" s="16" t="s">
-        <v>1437</v>
+        <v>1436</v>
       </c>
       <c r="B77" s="3" t="s">
         <v>451</v>
@@ -8306,7 +8306,7 @@
     </row>
     <row r="78" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A78" s="16" t="s">
-        <v>1438</v>
+        <v>1437</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>475</v>
@@ -8345,7 +8345,7 @@
     </row>
     <row r="79" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A79" s="16" t="s">
-        <v>1439</v>
+        <v>1438</v>
       </c>
       <c r="B79" s="3" t="s">
         <v>481</v>
@@ -8384,7 +8384,7 @@
     </row>
     <row r="80" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A80" s="16" t="s">
-        <v>1440</v>
+        <v>1439</v>
       </c>
       <c r="B80" s="3" t="s">
         <v>14</v>
@@ -8423,7 +8423,7 @@
     </row>
     <row r="81" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A81" s="16" t="s">
-        <v>1441</v>
+        <v>1440</v>
       </c>
       <c r="B81" s="3" t="s">
         <v>492</v>
@@ -8462,7 +8462,7 @@
     </row>
     <row r="82" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A82" s="16" t="s">
-        <v>1442</v>
+        <v>1441</v>
       </c>
       <c r="B82" s="3" t="s">
         <v>498</v>
@@ -8501,7 +8501,7 @@
     </row>
     <row r="83" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A83" s="16" t="s">
-        <v>1443</v>
+        <v>1442</v>
       </c>
       <c r="B83" s="3" t="s">
         <v>504</v>
@@ -8540,7 +8540,7 @@
     </row>
     <row r="84" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A84" s="16" t="s">
-        <v>1444</v>
+        <v>1443</v>
       </c>
       <c r="B84" s="3" t="s">
         <v>56</v>
@@ -8579,7 +8579,7 @@
     </row>
     <row r="85" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A85" s="16" t="s">
-        <v>1445</v>
+        <v>1444</v>
       </c>
       <c r="B85" s="3" t="s">
         <v>514</v>
@@ -8618,7 +8618,7 @@
     </row>
     <row r="86" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A86" s="16" t="s">
-        <v>1446</v>
+        <v>1445</v>
       </c>
       <c r="B86" s="3" t="s">
         <v>520</v>
@@ -8657,7 +8657,7 @@
     </row>
     <row r="87" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A87" s="16" t="s">
-        <v>1447</v>
+        <v>1446</v>
       </c>
       <c r="B87" s="3" t="s">
         <v>525</v>
@@ -8696,7 +8696,7 @@
     </row>
     <row r="88" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A88" s="16" t="s">
-        <v>1448</v>
+        <v>1447</v>
       </c>
       <c r="B88" s="3" t="s">
         <v>56</v>
@@ -8774,7 +8774,7 @@
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A90" s="16" t="s">
-        <v>1449</v>
+        <v>1448</v>
       </c>
       <c r="B90" s="3" t="s">
         <v>547</v>
@@ -8813,7 +8813,7 @@
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A91" s="16" t="s">
-        <v>1450</v>
+        <v>1449</v>
       </c>
       <c r="B91" s="3" t="s">
         <v>553</v>
@@ -8852,7 +8852,7 @@
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A92" s="16" t="s">
-        <v>1451</v>
+        <v>1450</v>
       </c>
       <c r="B92" s="3" t="s">
         <v>560</v>
@@ -8891,7 +8891,7 @@
     </row>
     <row r="93" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A93" s="16" t="s">
-        <v>1452</v>
+        <v>1451</v>
       </c>
       <c r="B93" s="3" t="s">
         <v>14</v>
@@ -8930,7 +8930,7 @@
     </row>
     <row r="94" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A94" s="16" t="s">
-        <v>1453</v>
+        <v>1452</v>
       </c>
       <c r="B94" s="3" t="s">
         <v>46</v>
@@ -8969,7 +8969,7 @@
     </row>
     <row r="95" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A95" s="16" t="s">
-        <v>1454</v>
+        <v>1453</v>
       </c>
       <c r="B95" s="3" t="s">
         <v>14</v>
@@ -9008,7 +9008,7 @@
     </row>
     <row r="96" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A96" s="16" t="s">
-        <v>1455</v>
+        <v>1454</v>
       </c>
       <c r="B96" s="3" t="s">
         <v>194</v>
@@ -9047,7 +9047,7 @@
     </row>
     <row r="97" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A97" s="16" t="s">
-        <v>1456</v>
+        <v>1455</v>
       </c>
       <c r="B97" s="3" t="s">
         <v>584</v>
@@ -9125,7 +9125,7 @@
     </row>
     <row r="99" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A99" s="16" t="s">
-        <v>1457</v>
+        <v>1456</v>
       </c>
       <c r="B99" s="3" t="s">
         <v>593</v>
@@ -9164,7 +9164,7 @@
     </row>
     <row r="100" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A100" s="16" t="s">
-        <v>1458</v>
+        <v>1457</v>
       </c>
       <c r="B100" s="3" t="s">
         <v>599</v>
@@ -9203,7 +9203,7 @@
     </row>
     <row r="101" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A101" s="16" t="s">
-        <v>1459</v>
+        <v>1458</v>
       </c>
       <c r="B101" s="3" t="s">
         <v>606</v>
@@ -9242,7 +9242,7 @@
     </row>
     <row r="102" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A102" s="16" t="s">
-        <v>1460</v>
+        <v>1459</v>
       </c>
       <c r="B102" s="3" t="s">
         <v>611</v>
@@ -9281,7 +9281,7 @@
     </row>
     <row r="103" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A103" s="16" t="s">
-        <v>1461</v>
+        <v>1460</v>
       </c>
       <c r="B103" s="3" t="s">
         <v>617</v>
@@ -9320,7 +9320,7 @@
     </row>
     <row r="104" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A104" s="16" t="s">
-        <v>1462</v>
+        <v>1461</v>
       </c>
       <c r="B104" s="3" t="s">
         <v>622</v>
@@ -9359,7 +9359,7 @@
     </row>
     <row r="105" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A105" s="16" t="s">
-        <v>1463</v>
+        <v>1462</v>
       </c>
       <c r="B105" s="3" t="s">
         <v>26</v>
@@ -9398,7 +9398,7 @@
     </row>
     <row r="106" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A106" s="16" t="s">
-        <v>1464</v>
+        <v>1463</v>
       </c>
       <c r="B106" s="3" t="s">
         <v>634</v>
@@ -9437,7 +9437,7 @@
     </row>
     <row r="107" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A107" s="16" t="s">
-        <v>1465</v>
+        <v>1464</v>
       </c>
       <c r="B107" s="3" t="s">
         <v>14</v>
@@ -9476,7 +9476,7 @@
     </row>
     <row r="108" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A108" s="16" t="s">
-        <v>1466</v>
+        <v>1465</v>
       </c>
       <c r="B108" s="3" t="s">
         <v>451</v>
@@ -9515,7 +9515,7 @@
     </row>
     <row r="109" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A109" s="16" t="s">
-        <v>1467</v>
+        <v>1466</v>
       </c>
       <c r="B109" s="3" t="s">
         <v>56</v>
@@ -9595,7 +9595,7 @@
     </row>
     <row r="111" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A111" s="16" t="s">
-        <v>1468</v>
+        <v>1552</v>
       </c>
       <c r="B111" s="3" t="s">
         <v>652</v>
@@ -9673,7 +9673,7 @@
     </row>
     <row r="113" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A113" s="16" t="s">
-        <v>1469</v>
+        <v>1467</v>
       </c>
       <c r="B113" s="3" t="s">
         <v>661</v>
@@ -9712,7 +9712,7 @@
     </row>
     <row r="114" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A114" s="16" t="s">
-        <v>1470</v>
+        <v>1468</v>
       </c>
       <c r="B114" s="3" t="s">
         <v>667</v>
@@ -9751,7 +9751,7 @@
     </row>
     <row r="115" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A115" s="16" t="s">
-        <v>1471</v>
+        <v>1469</v>
       </c>
       <c r="B115" s="3" t="s">
         <v>41</v>
@@ -9790,7 +9790,7 @@
     </row>
     <row r="116" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A116" s="16" t="s">
-        <v>1472</v>
+        <v>1470</v>
       </c>
       <c r="B116" s="3" t="s">
         <v>676</v>
@@ -9829,7 +9829,7 @@
     </row>
     <row r="117" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A117" s="16" t="s">
-        <v>1473</v>
+        <v>1471</v>
       </c>
       <c r="B117" s="3" t="s">
         <v>46</v>
@@ -9868,7 +9868,7 @@
     </row>
     <row r="118" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A118" s="16" t="s">
-        <v>1474</v>
+        <v>1472</v>
       </c>
       <c r="B118" s="3" t="s">
         <v>687</v>
@@ -9907,7 +9907,7 @@
     </row>
     <row r="119" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A119" s="16" t="s">
-        <v>1475</v>
+        <v>1473</v>
       </c>
       <c r="B119" s="3" t="s">
         <v>692</v>
@@ -9946,7 +9946,7 @@
     </row>
     <row r="120" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A120" s="16" t="s">
-        <v>1476</v>
+        <v>1474</v>
       </c>
       <c r="B120" s="3" t="s">
         <v>698</v>
@@ -9985,7 +9985,7 @@
     </row>
     <row r="121" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A121" s="16" t="s">
-        <v>1477</v>
+        <v>1475</v>
       </c>
       <c r="B121" s="3" t="s">
         <v>56</v>
@@ -10024,7 +10024,7 @@
     </row>
     <row r="122" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A122" s="16" t="s">
-        <v>1478</v>
+        <v>1476</v>
       </c>
       <c r="B122" s="3" t="s">
         <v>709</v>
@@ -10063,7 +10063,7 @@
     </row>
     <row r="123" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A123" s="16" t="s">
-        <v>1479</v>
+        <v>1477</v>
       </c>
       <c r="B123" s="3" t="s">
         <v>113</v>
@@ -10102,7 +10102,7 @@
     </row>
     <row r="124" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A124" s="16" t="s">
-        <v>1480</v>
+        <v>1478</v>
       </c>
       <c r="B124" s="3" t="s">
         <v>46</v>
@@ -10141,7 +10141,7 @@
     </row>
     <row r="125" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A125" s="16" t="s">
-        <v>1481</v>
+        <v>1479</v>
       </c>
       <c r="B125" s="3" t="s">
         <v>723</v>
@@ -10180,7 +10180,7 @@
     </row>
     <row r="126" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A126" s="16" t="s">
-        <v>1482</v>
+        <v>1480</v>
       </c>
       <c r="B126" s="3" t="s">
         <v>728</v>
@@ -10219,7 +10219,7 @@
     </row>
     <row r="127" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A127" s="16" t="s">
-        <v>1483</v>
+        <v>1481</v>
       </c>
       <c r="B127" s="3" t="s">
         <v>734</v>
@@ -10258,7 +10258,7 @@
     </row>
     <row r="128" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A128" s="16" t="s">
-        <v>1484</v>
+        <v>1482</v>
       </c>
       <c r="B128" s="3" t="s">
         <v>14</v>
@@ -10297,7 +10297,7 @@
     </row>
     <row r="129" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A129" s="16" t="s">
-        <v>1485</v>
+        <v>1483</v>
       </c>
       <c r="B129" s="3" t="s">
         <v>194</v>
@@ -10336,7 +10336,7 @@
     </row>
     <row r="130" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A130" s="16" t="s">
-        <v>1486</v>
+        <v>1484</v>
       </c>
       <c r="B130" s="3" t="s">
         <v>744</v>
@@ -10375,7 +10375,7 @@
     </row>
     <row r="131" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A131" s="16" t="s">
-        <v>1487</v>
+        <v>1485</v>
       </c>
       <c r="B131" s="3" t="s">
         <v>748</v>
@@ -10414,7 +10414,7 @@
     </row>
     <row r="132" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A132" s="16" t="s">
-        <v>1488</v>
+        <v>1553</v>
       </c>
       <c r="B132" s="3" t="s">
         <v>14</v>
@@ -10454,7 +10454,7 @@
     </row>
     <row r="133" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A133" s="16" t="s">
-        <v>1489</v>
+        <v>1486</v>
       </c>
       <c r="B133" s="3" t="s">
         <v>754</v>
@@ -10493,7 +10493,7 @@
     </row>
     <row r="134" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A134" s="16" t="s">
-        <v>1490</v>
+        <v>1487</v>
       </c>
       <c r="B134" s="3" t="s">
         <v>56</v>
@@ -10532,7 +10532,7 @@
     </row>
     <row r="135" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A135" s="16" t="s">
-        <v>1491</v>
+        <v>1488</v>
       </c>
       <c r="B135" s="3" t="s">
         <v>764</v>
@@ -10571,7 +10571,7 @@
     </row>
     <row r="136" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A136" s="16" t="s">
-        <v>1492</v>
+        <v>1489</v>
       </c>
       <c r="B136" s="3" t="s">
         <v>771</v>
@@ -10610,7 +10610,7 @@
     </row>
     <row r="137" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A137" s="16" t="s">
-        <v>1493</v>
+        <v>1490</v>
       </c>
       <c r="B137" s="3" t="s">
         <v>123</v>
@@ -10649,7 +10649,7 @@
     </row>
     <row r="138" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A138" s="16" t="s">
-        <v>1494</v>
+        <v>1491</v>
       </c>
       <c r="B138" s="3" t="s">
         <v>781</v>
@@ -10688,7 +10688,7 @@
     </row>
     <row r="139" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A139" s="16" t="s">
-        <v>1495</v>
+        <v>1492</v>
       </c>
       <c r="B139" s="3" t="s">
         <v>788</v>
@@ -10727,7 +10727,7 @@
     </row>
     <row r="140" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A140" s="16" t="s">
-        <v>1496</v>
+        <v>1493</v>
       </c>
       <c r="B140" s="3" t="s">
         <v>41</v>
@@ -10766,7 +10766,7 @@
     </row>
     <row r="141" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A141" s="16" t="s">
-        <v>1497</v>
+        <v>1494</v>
       </c>
       <c r="B141" s="3" t="s">
         <v>797</v>
@@ -10805,7 +10805,7 @@
     </row>
     <row r="142" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A142" s="16" t="s">
-        <v>1498</v>
+        <v>1495</v>
       </c>
       <c r="B142" s="3" t="s">
         <v>801</v>
@@ -10844,7 +10844,7 @@
     </row>
     <row r="143" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A143" s="16" t="s">
-        <v>1499</v>
+        <v>1496</v>
       </c>
       <c r="B143" s="3" t="s">
         <v>652</v>
@@ -10883,7 +10883,7 @@
     </row>
     <row r="144" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A144" s="16" t="s">
-        <v>1500</v>
+        <v>1497</v>
       </c>
       <c r="B144" s="3" t="s">
         <v>812</v>
@@ -10922,7 +10922,7 @@
     </row>
     <row r="145" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A145" s="16" t="s">
-        <v>1501</v>
+        <v>1498</v>
       </c>
       <c r="B145" s="3" t="s">
         <v>46</v>
@@ -10961,7 +10961,7 @@
     </row>
     <row r="146" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A146" s="16" t="s">
-        <v>1502</v>
+        <v>1499</v>
       </c>
       <c r="B146" s="3" t="s">
         <v>46</v>
@@ -11000,7 +11000,7 @@
     </row>
     <row r="147" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A147" s="16" t="s">
-        <v>1503</v>
+        <v>1500</v>
       </c>
       <c r="B147" s="3" t="s">
         <v>829</v>
@@ -11078,7 +11078,7 @@
     </row>
     <row r="149" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A149" s="16" t="s">
-        <v>1504</v>
+        <v>1501</v>
       </c>
       <c r="B149" s="3" t="s">
         <v>41</v>
@@ -11117,7 +11117,7 @@
     </row>
     <row r="150" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A150" s="16" t="s">
-        <v>1505</v>
+        <v>1502</v>
       </c>
       <c r="B150" s="3" t="s">
         <v>14</v>
@@ -11156,7 +11156,7 @@
     </row>
     <row r="151" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A151" s="16" t="s">
-        <v>1506</v>
+        <v>1503</v>
       </c>
       <c r="B151" s="3" t="s">
         <v>848</v>
@@ -11195,7 +11195,7 @@
     </row>
     <row r="152" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A152" s="16" t="s">
-        <v>1507</v>
+        <v>1504</v>
       </c>
       <c r="B152" s="3" t="s">
         <v>896</v>
@@ -11234,7 +11234,7 @@
     </row>
     <row r="153" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A153" s="16" t="s">
-        <v>1508</v>
+        <v>1505</v>
       </c>
       <c r="B153" s="3" t="s">
         <v>113</v>
@@ -11273,7 +11273,7 @@
     </row>
     <row r="154" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A154" s="16" t="s">
-        <v>1509</v>
+        <v>1506</v>
       </c>
       <c r="B154" s="3" t="s">
         <v>905</v>
@@ -11312,7 +11312,7 @@
     </row>
     <row r="155" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A155" s="16" t="s">
-        <v>1510</v>
+        <v>1507</v>
       </c>
       <c r="B155" s="3" t="s">
         <v>910</v>
@@ -11351,7 +11351,7 @@
     </row>
     <row r="156" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A156" s="16" t="s">
-        <v>1511</v>
+        <v>1508</v>
       </c>
       <c r="B156" s="3" t="s">
         <v>46</v>
@@ -11390,7 +11390,7 @@
     </row>
     <row r="157" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A157" s="16" t="s">
-        <v>1512</v>
+        <v>1509</v>
       </c>
       <c r="B157" s="3" t="s">
         <v>923</v>
@@ -11468,7 +11468,7 @@
     </row>
     <row r="159" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A159" s="16" t="s">
-        <v>1513</v>
+        <v>1510</v>
       </c>
       <c r="B159" s="3" t="s">
         <v>933</v>
@@ -11507,7 +11507,7 @@
     </row>
     <row r="160" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A160" s="16" t="s">
-        <v>1514</v>
+        <v>1511</v>
       </c>
       <c r="B160" s="3" t="s">
         <v>938</v>
@@ -11546,7 +11546,7 @@
     </row>
     <row r="161" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A161" s="16" t="s">
-        <v>1515</v>
+        <v>1512</v>
       </c>
       <c r="B161" s="3" t="s">
         <v>943</v>
@@ -11585,7 +11585,7 @@
     </row>
     <row r="162" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A162" s="16" t="s">
-        <v>1516</v>
+        <v>1513</v>
       </c>
       <c r="B162" s="3" t="s">
         <v>56</v>
@@ -11624,7 +11624,7 @@
     </row>
     <row r="163" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A163" s="16" t="s">
-        <v>1517</v>
+        <v>1514</v>
       </c>
       <c r="B163" s="3" t="s">
         <v>953</v>
@@ -11663,7 +11663,7 @@
     </row>
     <row r="164" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A164" s="16" t="s">
-        <v>1518</v>
+        <v>1515</v>
       </c>
       <c r="B164" s="3" t="s">
         <v>46</v>
@@ -11702,7 +11702,7 @@
     </row>
     <row r="165" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A165" s="16" t="s">
-        <v>1519</v>
+        <v>1516</v>
       </c>
       <c r="B165" s="3" t="s">
         <v>46</v>
@@ -11741,7 +11741,7 @@
     </row>
     <row r="166" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A166" s="16" t="s">
-        <v>1520</v>
+        <v>1517</v>
       </c>
       <c r="B166" s="3" t="s">
         <v>46</v>
@@ -11780,7 +11780,7 @@
     </row>
     <row r="167" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A167" s="16" t="s">
-        <v>1521</v>
+        <v>1518</v>
       </c>
       <c r="B167" s="3" t="s">
         <v>971</v>
@@ -11819,7 +11819,7 @@
     </row>
     <row r="168" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A168" s="16" t="s">
-        <v>1522</v>
+        <v>1519</v>
       </c>
       <c r="B168" s="3" t="s">
         <v>976</v>
@@ -11858,7 +11858,7 @@
     </row>
     <row r="169" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A169" s="16" t="s">
-        <v>1523</v>
+        <v>1520</v>
       </c>
       <c r="B169" s="3" t="s">
         <v>723</v>
@@ -11897,7 +11897,7 @@
     </row>
     <row r="170" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A170" s="16" t="s">
-        <v>1524</v>
+        <v>1521</v>
       </c>
       <c r="B170" s="3" t="s">
         <v>46</v>
@@ -11936,7 +11936,7 @@
     </row>
     <row r="171" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A171" s="16" t="s">
-        <v>1525</v>
+        <v>1522</v>
       </c>
       <c r="B171" s="3" t="s">
         <v>709</v>
@@ -11975,7 +11975,7 @@
     </row>
     <row r="172" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A172" s="16" t="s">
-        <v>1526</v>
+        <v>1523</v>
       </c>
       <c r="B172" s="3" t="s">
         <v>14</v>
@@ -12014,7 +12014,7 @@
     </row>
     <row r="173" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A173" s="16" t="s">
-        <v>1527</v>
+        <v>1524</v>
       </c>
       <c r="B173" s="3" t="s">
         <v>1001</v>
@@ -12092,7 +12092,7 @@
     </row>
     <row r="175" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A175" s="16" t="s">
-        <v>1528</v>
+        <v>1525</v>
       </c>
       <c r="B175" s="3" t="s">
         <v>492</v>
@@ -12131,7 +12131,7 @@
     </row>
     <row r="176" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A176" s="16" t="s">
-        <v>1529</v>
+        <v>1526</v>
       </c>
       <c r="B176" s="3" t="s">
         <v>1013</v>
@@ -12170,7 +12170,7 @@
     </row>
     <row r="177" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A177" s="16" t="s">
-        <v>1530</v>
+        <v>1527</v>
       </c>
       <c r="B177" s="3" t="s">
         <v>1019</v>
@@ -12209,7 +12209,7 @@
     </row>
     <row r="178" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A178" s="16" t="s">
-        <v>1531</v>
+        <v>1528</v>
       </c>
       <c r="B178" s="3" t="s">
         <v>1024</v>
@@ -12248,7 +12248,7 @@
     </row>
     <row r="179" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A179" s="16" t="s">
-        <v>1532</v>
+        <v>1529</v>
       </c>
       <c r="B179" s="3" t="s">
         <v>46</v>
@@ -12287,7 +12287,7 @@
     </row>
     <row r="180" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A180" s="16" t="s">
-        <v>1533</v>
+        <v>1530</v>
       </c>
       <c r="B180" s="3" t="s">
         <v>1036</v>
@@ -12326,7 +12326,7 @@
     </row>
     <row r="181" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A181" s="16" t="s">
-        <v>1534</v>
+        <v>1531</v>
       </c>
       <c r="B181" s="3" t="s">
         <v>1041</v>
@@ -12365,7 +12365,7 @@
     </row>
     <row r="182" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A182" s="16" t="s">
-        <v>1535</v>
+        <v>1532</v>
       </c>
       <c r="B182" s="3" t="s">
         <v>14</v>
@@ -12404,7 +12404,7 @@
     </row>
     <row r="183" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A183" s="16" t="s">
-        <v>1536</v>
+        <v>1533</v>
       </c>
       <c r="B183" s="3" t="s">
         <v>1052</v>
@@ -12443,7 +12443,7 @@
     </row>
     <row r="184" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A184" s="16" t="s">
-        <v>1537</v>
+        <v>1534</v>
       </c>
       <c r="B184" s="3" t="s">
         <v>1058</v>
@@ -12482,7 +12482,7 @@
     </row>
     <row r="185" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A185" s="16" t="s">
-        <v>1538</v>
+        <v>1535</v>
       </c>
       <c r="B185" s="3" t="s">
         <v>1064</v>
@@ -12521,7 +12521,7 @@
     </row>
     <row r="186" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A186" s="16" t="s">
-        <v>1539</v>
+        <v>1536</v>
       </c>
       <c r="B186" s="3" t="s">
         <v>492</v>
@@ -12560,7 +12560,7 @@
     </row>
     <row r="187" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A187" s="16" t="s">
-        <v>1540</v>
+        <v>1537</v>
       </c>
       <c r="B187" s="3" t="s">
         <v>1075</v>
@@ -12599,7 +12599,7 @@
     </row>
     <row r="188" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A188" s="16" t="s">
-        <v>1541</v>
+        <v>1538</v>
       </c>
       <c r="B188" s="3" t="s">
         <v>1080</v>
@@ -12638,7 +12638,7 @@
     </row>
     <row r="189" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A189" s="16" t="s">
-        <v>1542</v>
+        <v>1539</v>
       </c>
       <c r="B189" s="3" t="s">
         <v>56</v>
@@ -12677,7 +12677,7 @@
     </row>
     <row r="190" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A190" s="16" t="s">
-        <v>1543</v>
+        <v>1540</v>
       </c>
       <c r="B190" s="3" t="s">
         <v>1081</v>
@@ -12716,7 +12716,7 @@
     </row>
     <row r="191" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A191" s="16" t="s">
-        <v>1544</v>
+        <v>1541</v>
       </c>
       <c r="B191" s="3" t="s">
         <v>1098</v>
@@ -12755,7 +12755,7 @@
     </row>
     <row r="192" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A192" s="16" t="s">
-        <v>1545</v>
+        <v>1542</v>
       </c>
       <c r="B192" s="3" t="s">
         <v>1104</v>
@@ -12794,7 +12794,7 @@
     </row>
     <row r="193" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A193" s="16" t="s">
-        <v>1546</v>
+        <v>1543</v>
       </c>
       <c r="B193" s="3" t="s">
         <v>56</v>
@@ -12833,7 +12833,7 @@
     </row>
     <row r="194" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A194" s="16" t="s">
-        <v>1547</v>
+        <v>1544</v>
       </c>
       <c r="B194" s="3" t="s">
         <v>14</v>
@@ -12872,7 +12872,7 @@
     </row>
     <row r="195" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A195" s="16" t="s">
-        <v>1548</v>
+        <v>1545</v>
       </c>
       <c r="B195" s="3" t="s">
         <v>46</v>
@@ -12911,7 +12911,7 @@
     </row>
     <row r="196" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A196" s="16" t="s">
-        <v>1549</v>
+        <v>1546</v>
       </c>
       <c r="B196" s="3" t="s">
         <v>46</v>
@@ -12950,7 +12950,7 @@
     </row>
     <row r="197" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A197" s="16" t="s">
-        <v>1550</v>
+        <v>1547</v>
       </c>
       <c r="B197" s="3" t="s">
         <v>1127</v>
@@ -13028,7 +13028,7 @@
     </row>
     <row r="199" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A199" s="16" t="s">
-        <v>1551</v>
+        <v>1548</v>
       </c>
       <c r="B199" s="3" t="s">
         <v>1139</v>
@@ -13067,7 +13067,7 @@
     </row>
     <row r="200" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A200" s="16" t="s">
-        <v>1552</v>
+        <v>1550</v>
       </c>
       <c r="B200" s="3" t="s">
         <v>1144</v>

</xml_diff>